<commit_message>
Name the shop SAPTHAGIRI PARTY SHOP and fit the name on phone screens
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FgoJdnchEhiY3W9DSyRdxS
</commit_message>
<xml_diff>
--- a/decor-shop/sheet-template/Decor-Shop-Sheet.xlsx
+++ b/decor-shop/sheet-template/Decor-Shop-Sheet.xlsx
@@ -457,7 +457,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Your Shop Name</t>
+          <t>SAPTHAGIRI PARTY SHOP</t>
         </is>
       </c>
     </row>
@@ -469,7 +469,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Decorations for birthdays, baby showers and every festival — delivered to your door.</t>
+          <t>Party &amp; festival decorations for birthdays, baby showers, Diwali, Dussehra, Halloween, Christmas and every celebration.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add shop locations with maps, directions and pickup option
Shops are listed from a new Shops tab in the Google Sheet. Customers can
choose home delivery or pickup from a shop, and checkout details are kept
when cart quantities change.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FgoJdnchEhiY3W9DSyRdxS
</commit_message>
<xml_diff>
--- a/decor-shop/sheet-template/Decor-Shop-Sheet.xlsx
+++ b/decor-shop/sheet-template/Decor-Shop-Sheet.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Collections" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shops" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1029,4 +1030,114 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Address</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Map Link</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Timings</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Show</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>SAPTHAGIRI PARTY SHOP – Main Branch</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Shop address, Area, City – PIN</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>+91 98765 43210</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>10 AM – 9 PM, all days</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>SAPTHAGIRI PARTY SHOP – Branch 2</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Shop address, Area, City – PIN</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr"/>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>+91 98765 43210</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>10 AM – 9 PM, closed Tuesday</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add Sapthagiri contact details and the four shop locations
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FgoJdnchEhiY3W9DSyRdxS
</commit_message>
<xml_diff>
--- a/decor-shop/sheet-template/Decor-Shop-Sheet.xlsx
+++ b/decor-shop/sheet-template/Decor-Shop-Sheet.xlsx
@@ -482,7 +482,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>+91 98765 43210</t>
+          <t>+91 98808 55551</t>
         </is>
       </c>
     </row>
@@ -494,7 +494,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>yourshop@gmail.com</t>
+          <t>rakeshbabyls@gmail.com</t>
         </is>
       </c>
     </row>
@@ -506,7 +506,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>+91 98765 43210</t>
+          <t>+91 98808 55551</t>
         </is>
       </c>
     </row>
@@ -516,11 +516,7 @@
           <t>Address</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Shop no. 1, Main Market, Your City</t>
-        </is>
-      </c>
+      <c r="B7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -528,11 +524,7 @@
           <t>Instagram</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>@yourshop</t>
-        </is>
-      </c>
+      <c r="B8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1038,15 +1030,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="44" customWidth="1" min="2" max="2"/>
-    <col width="36" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1057,25 +1050,30 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>About</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Address</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Map Link</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Timings</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Show</t>
         </is>
@@ -1084,26 +1082,27 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>SAPTHAGIRI PARTY SHOP – Main Branch</t>
+          <t>Sapthagiri Party Shop</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Shop address, Area, City – PIN</t>
+          <t>Retail · Birthday · Halloween · Christmas</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr"/>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>+91 98765 43210</t>
+          <t>https://maps.app.goo.gl/Q5BkWGuxpkbWK8W49</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>10 AM – 9 PM, all days</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
+          <t>+91 98808 55551</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -1112,26 +1111,85 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>SAPTHAGIRI PARTY SHOP – Branch 2</t>
+          <t>Sapthagiri Party Shop – Main Outlet</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Shop address, Area, City – PIN</t>
+          <t>Our main outlet</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr"/>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>+91 98765 43210</t>
+          <t>https://maps.app.goo.gl/3qZwUjtAYMwjRRey9</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>10 AM – 9 PM, closed Tuesday</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
+          <t>+91 98808 55551</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr"/>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Sapthagiri Regalia</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Birthday decorations – main store</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>https://maps.app.goo.gl/3CZ5u6ptdbV4ymMu5</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>+91 98808 55551</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr"/>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Vishnu Enterprises</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Event decor</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr"/>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>https://maps.app.goo.gl/GiXUgLquWgZUhxhR6</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>+91 98808 55551</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr"/>
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>

</xml_diff>

<commit_message>
Send shop pickup orders to that shop's WhatsApp numbers as well as the main number
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FgoJdnchEhiY3W9DSyRdxS
</commit_message>
<xml_diff>
--- a/decor-shop/sheet-template/Decor-Shop-Sheet.xlsx
+++ b/decor-shop/sheet-template/Decor-Shop-Sheet.xlsx
@@ -1030,16 +1030,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="36" customWidth="1" min="2" max="2"/>
     <col width="40" customWidth="1" min="3" max="3"/>
     <col width="44" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1065,15 +1066,20 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Timings</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Show</t>
         </is>
@@ -1098,11 +1104,16 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>+91 98808 55551</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr">
+          <t>+91 98861 80607</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>+91 98861 80607</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -1127,11 +1138,16 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>+91 98808 55551</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr"/>
-      <c r="G3" s="2" t="inlineStr">
+          <t>+91 98802 02339</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>+91 98802 02339</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -1156,11 +1172,16 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>+91 98808 55551</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr"/>
-      <c r="G4" s="2" t="inlineStr">
+          <t>+91 96208 19550</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>+91 96208 19550</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -1185,11 +1206,16 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>+91 98808 55551</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr"/>
-      <c r="G5" s="2" t="inlineStr">
+          <t>+91 96636 23051</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>+91 96636 23051</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>

</xml_diff>